<commit_message>
Added v3.0.0 strings in order to ease the merge
</commit_message>
<xml_diff>
--- a/translations/translations.xlsx
+++ b/translations/translations.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/russell/Projects/GPS-Sample/translations/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E1114FC5-7AEF-4844-9F4C-A5580B57DC9B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{21A62F6D-B106-AC40-9AA4-C84BCFCDBDFB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17740" xr2:uid="{C8C8ACD1-4E76-7942-B525-8D880B4ECA80}"/>
+    <workbookView xWindow="7960" yWindow="800" windowWidth="30240" windowHeight="22740" xr2:uid="{C8C8ACD1-4E76-7942-B525-8D880B4ECA80}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -67,7 +67,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5430" uniqueCount="5068">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5474" uniqueCount="5112">
   <si>
     <t>app_name</t>
   </si>
@@ -15271,13 +15271,145 @@
   </si>
   <si>
     <t>واټن</t>
+  </si>
+  <si>
+    <t>enforce_geofence_boundary</t>
+  </si>
+  <si>
+    <t>enter_the_geofence_buffer_value</t>
+  </si>
+  <si>
+    <t>geofence_hint</t>
+  </si>
+  <si>
+    <t>geofence_error</t>
+  </si>
+  <si>
+    <t>begin_sample_review</t>
+  </si>
+  <si>
+    <t>review_sample</t>
+  </si>
+  <si>
+    <t>review_possible_duplicates</t>
+  </si>
+  <si>
+    <t>review_boundary_violations</t>
+  </si>
+  <si>
+    <t>save_sample</t>
+  </si>
+  <si>
+    <t>duplicate</t>
+  </si>
+  <si>
+    <t>outside_boundary</t>
+  </si>
+  <si>
+    <t>reason_is_required</t>
+  </si>
+  <si>
+    <t>location</t>
+  </si>
+  <si>
+    <t>keep_or_exclude_this_location</t>
+  </si>
+  <si>
+    <t>keep_this_location</t>
+  </si>
+  <si>
+    <t>exclude_this_location</t>
+  </si>
+  <si>
+    <t>reason</t>
+  </si>
+  <si>
+    <t>delete_location_message</t>
+  </si>
+  <si>
+    <t>open</t>
+  </si>
+  <si>
+    <t>edit</t>
+  </si>
+  <si>
+    <t>clone</t>
+  </si>
+  <si>
+    <t>configuration</t>
+  </si>
+  <si>
+    <t>Enforce Geofence Boundary</t>
+  </si>
+  <si>
+    <t>Enter the geofence buffer value</t>
+  </si>
+  <si>
+    <t>Placeholder for GeoFence Hint</t>
+  </si>
+  <si>
+    <t>You are currently outside of the Geofence</t>
+  </si>
+  <si>
+    <t>Begin Sample Review</t>
+  </si>
+  <si>
+    <t>Review Sample</t>
+  </si>
+  <si>
+    <t>Review Possible Duplicates</t>
+  </si>
+  <si>
+    <t>Review Boundary Violations</t>
+  </si>
+  <si>
+    <t>Save Sample</t>
+  </si>
+  <si>
+    <t>Duplicate</t>
+  </si>
+  <si>
+    <t>Outside Boundary</t>
+  </si>
+  <si>
+    <t>You must select a Reason for the exclusion.</t>
+  </si>
+  <si>
+    <t>Location</t>
+  </si>
+  <si>
+    <t>Keep or Exclude this location?</t>
+  </si>
+  <si>
+    <t>Keep this location</t>
+  </si>
+  <si>
+    <t>Exclude this location</t>
+  </si>
+  <si>
+    <t>Reason</t>
+  </si>
+  <si>
+    <t>Would you also like to permanently delete this location?</t>
+  </si>
+  <si>
+    <t>Open</t>
+  </si>
+  <si>
+    <t>Edit</t>
+  </si>
+  <si>
+    <t>Clone</t>
+  </si>
+  <si>
+    <t>Configuration</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="12">
+  <fonts count="13">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -15360,6 +15492,13 @@
       <family val="2"/>
       <scheme val="major"/>
     </font>
+    <font>
+      <sz val="8"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri Light"/>
+      <family val="2"/>
+      <scheme val="major"/>
+    </font>
   </fonts>
   <fills count="8">
     <fill>
@@ -15405,7 +15544,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -15437,11 +15576,20 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="39">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -15525,6 +15673,20 @@
     <xf numFmtId="0" fontId="11" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -15746,8 +15908,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{73295AEA-8140-4EAB-A7A6-7D1875F4D7E7}" name="Table1" displayName="Table1" ref="A1:J543" totalsRowShown="0" headerRowDxfId="11" dataDxfId="10">
-  <autoFilter ref="A1:J543" xr:uid="{73295AEA-8140-4EAB-A7A6-7D1875F4D7E7}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{73295AEA-8140-4EAB-A7A6-7D1875F4D7E7}" name="Table1" displayName="Table1" ref="A1:J565" totalsRowShown="0" headerRowDxfId="11" dataDxfId="10">
+  <autoFilter ref="A1:J565" xr:uid="{73295AEA-8140-4EAB-A7A6-7D1875F4D7E7}"/>
   <tableColumns count="10">
     <tableColumn id="1" xr3:uid="{DE67F62A-9DCA-4DFE-8C98-83B024E5D946}" name="app_name" dataDxfId="9"/>
     <tableColumn id="2" xr3:uid="{BCDA3AB5-7BB5-4A21-ABBB-4186B52D559D}" name="GPSSample::en" dataDxfId="8"/>
@@ -16073,7 +16235,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8BD3E6CC-854C-5841-9577-D3ADD2982DB6}">
-  <dimension ref="A1:J543"/>
+  <dimension ref="A1:J565"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16"/>
   <cols>
     <col min="1" max="1" width="33.5" customWidth="1"/>
@@ -33461,6 +33623,358 @@
       <c r="J543" s="12" t="s">
         <v>5067</v>
       </c>
+    </row>
+    <row r="544" spans="1:10">
+      <c r="A544" s="33" t="s">
+        <v>5068</v>
+      </c>
+      <c r="B544" s="34" t="s">
+        <v>5090</v>
+      </c>
+      <c r="C544" s="35"/>
+      <c r="D544" s="35"/>
+      <c r="E544" s="35"/>
+      <c r="F544" s="35"/>
+      <c r="G544" s="36"/>
+      <c r="H544" s="35"/>
+      <c r="I544" s="37"/>
+      <c r="J544" s="37"/>
+    </row>
+    <row r="545" spans="1:10">
+      <c r="A545" s="33" t="s">
+        <v>5069</v>
+      </c>
+      <c r="B545" s="34" t="s">
+        <v>5091</v>
+      </c>
+      <c r="C545" s="35"/>
+      <c r="D545" s="35"/>
+      <c r="E545" s="35"/>
+      <c r="F545" s="35"/>
+      <c r="G545" s="36"/>
+      <c r="H545" s="35"/>
+      <c r="I545" s="37"/>
+      <c r="J545" s="37"/>
+    </row>
+    <row r="546" spans="1:10">
+      <c r="A546" s="33" t="s">
+        <v>5070</v>
+      </c>
+      <c r="B546" s="34" t="s">
+        <v>5092</v>
+      </c>
+      <c r="C546" s="35"/>
+      <c r="D546" s="35"/>
+      <c r="E546" s="35"/>
+      <c r="F546" s="35"/>
+      <c r="G546" s="36"/>
+      <c r="H546" s="35"/>
+      <c r="I546" s="37"/>
+      <c r="J546" s="37"/>
+    </row>
+    <row r="547" spans="1:10">
+      <c r="A547" s="33" t="s">
+        <v>5071</v>
+      </c>
+      <c r="B547" s="38" t="s">
+        <v>5093</v>
+      </c>
+      <c r="C547" s="35"/>
+      <c r="D547" s="35"/>
+      <c r="E547" s="35"/>
+      <c r="F547" s="35"/>
+      <c r="G547" s="36"/>
+      <c r="H547" s="35"/>
+      <c r="I547" s="37"/>
+      <c r="J547" s="37"/>
+    </row>
+    <row r="548" spans="1:10">
+      <c r="A548" s="33" t="s">
+        <v>5072</v>
+      </c>
+      <c r="B548" s="38" t="s">
+        <v>5094</v>
+      </c>
+      <c r="C548" s="35"/>
+      <c r="D548" s="35"/>
+      <c r="E548" s="35"/>
+      <c r="F548" s="35"/>
+      <c r="G548" s="36"/>
+      <c r="H548" s="35"/>
+      <c r="I548" s="37"/>
+      <c r="J548" s="37"/>
+    </row>
+    <row r="549" spans="1:10">
+      <c r="A549" s="33" t="s">
+        <v>5073</v>
+      </c>
+      <c r="B549" s="38" t="s">
+        <v>5095</v>
+      </c>
+      <c r="C549" s="35"/>
+      <c r="D549" s="35"/>
+      <c r="E549" s="35"/>
+      <c r="F549" s="35"/>
+      <c r="G549" s="36"/>
+      <c r="H549" s="35"/>
+      <c r="I549" s="37"/>
+      <c r="J549" s="37"/>
+    </row>
+    <row r="550" spans="1:10">
+      <c r="A550" s="33" t="s">
+        <v>5074</v>
+      </c>
+      <c r="B550" s="38" t="s">
+        <v>5096</v>
+      </c>
+      <c r="C550" s="35"/>
+      <c r="D550" s="35"/>
+      <c r="E550" s="35"/>
+      <c r="F550" s="35"/>
+      <c r="G550" s="36"/>
+      <c r="H550" s="35"/>
+      <c r="I550" s="37"/>
+      <c r="J550" s="37"/>
+    </row>
+    <row r="551" spans="1:10">
+      <c r="A551" s="33" t="s">
+        <v>5075</v>
+      </c>
+      <c r="B551" s="38" t="s">
+        <v>5097</v>
+      </c>
+      <c r="C551" s="35"/>
+      <c r="D551" s="35"/>
+      <c r="E551" s="35"/>
+      <c r="F551" s="35"/>
+      <c r="G551" s="36"/>
+      <c r="H551" s="35"/>
+      <c r="I551" s="37"/>
+      <c r="J551" s="37"/>
+    </row>
+    <row r="552" spans="1:10">
+      <c r="A552" s="33" t="s">
+        <v>5076</v>
+      </c>
+      <c r="B552" s="38" t="s">
+        <v>5098</v>
+      </c>
+      <c r="C552" s="35"/>
+      <c r="D552" s="35"/>
+      <c r="E552" s="35"/>
+      <c r="F552" s="35"/>
+      <c r="G552" s="36"/>
+      <c r="H552" s="35"/>
+      <c r="I552" s="37"/>
+      <c r="J552" s="37"/>
+    </row>
+    <row r="553" spans="1:10">
+      <c r="A553" s="33" t="s">
+        <v>5077</v>
+      </c>
+      <c r="B553" s="34" t="s">
+        <v>5099</v>
+      </c>
+      <c r="C553" s="35"/>
+      <c r="D553" s="35"/>
+      <c r="E553" s="35"/>
+      <c r="F553" s="35"/>
+      <c r="G553" s="36"/>
+      <c r="H553" s="35"/>
+      <c r="I553" s="37"/>
+      <c r="J553" s="37"/>
+    </row>
+    <row r="554" spans="1:10">
+      <c r="A554" s="33" t="s">
+        <v>5078</v>
+      </c>
+      <c r="B554" s="34" t="s">
+        <v>5100</v>
+      </c>
+      <c r="C554" s="35"/>
+      <c r="D554" s="35"/>
+      <c r="E554" s="35"/>
+      <c r="F554" s="35"/>
+      <c r="G554" s="36"/>
+      <c r="H554" s="35"/>
+      <c r="I554" s="37"/>
+      <c r="J554" s="37"/>
+    </row>
+    <row r="555" spans="1:10">
+      <c r="A555" s="33" t="s">
+        <v>5079</v>
+      </c>
+      <c r="B555" s="38" t="s">
+        <v>5101</v>
+      </c>
+      <c r="C555" s="35"/>
+      <c r="D555" s="35"/>
+      <c r="E555" s="35"/>
+      <c r="F555" s="35"/>
+      <c r="G555" s="36"/>
+      <c r="H555" s="35"/>
+      <c r="I555" s="37"/>
+      <c r="J555" s="37"/>
+    </row>
+    <row r="556" spans="1:10">
+      <c r="A556" s="33" t="s">
+        <v>5080</v>
+      </c>
+      <c r="B556" s="34" t="s">
+        <v>5102</v>
+      </c>
+      <c r="C556" s="35"/>
+      <c r="D556" s="35"/>
+      <c r="E556" s="35"/>
+      <c r="F556" s="35"/>
+      <c r="G556" s="36"/>
+      <c r="H556" s="35"/>
+      <c r="I556" s="37"/>
+      <c r="J556" s="37"/>
+    </row>
+    <row r="557" spans="1:10">
+      <c r="A557" s="33" t="s">
+        <v>5081</v>
+      </c>
+      <c r="B557" s="34" t="s">
+        <v>5103</v>
+      </c>
+      <c r="C557" s="35"/>
+      <c r="D557" s="35"/>
+      <c r="E557" s="35"/>
+      <c r="F557" s="35"/>
+      <c r="G557" s="36"/>
+      <c r="H557" s="35"/>
+      <c r="I557" s="37"/>
+      <c r="J557" s="37"/>
+    </row>
+    <row r="558" spans="1:10">
+      <c r="A558" s="33" t="s">
+        <v>5082</v>
+      </c>
+      <c r="B558" s="34" t="s">
+        <v>5104</v>
+      </c>
+      <c r="C558" s="35"/>
+      <c r="D558" s="35"/>
+      <c r="E558" s="35"/>
+      <c r="F558" s="35"/>
+      <c r="G558" s="36"/>
+      <c r="H558" s="35"/>
+      <c r="I558" s="37"/>
+      <c r="J558" s="37"/>
+    </row>
+    <row r="559" spans="1:10">
+      <c r="A559" s="33" t="s">
+        <v>5083</v>
+      </c>
+      <c r="B559" s="34" t="s">
+        <v>5105</v>
+      </c>
+      <c r="C559" s="35"/>
+      <c r="D559" s="35"/>
+      <c r="E559" s="35"/>
+      <c r="F559" s="35"/>
+      <c r="G559" s="36"/>
+      <c r="H559" s="35"/>
+      <c r="I559" s="37"/>
+      <c r="J559" s="37"/>
+    </row>
+    <row r="560" spans="1:10">
+      <c r="A560" s="33" t="s">
+        <v>5084</v>
+      </c>
+      <c r="B560" s="34" t="s">
+        <v>5106</v>
+      </c>
+      <c r="C560" s="35"/>
+      <c r="D560" s="35"/>
+      <c r="E560" s="35"/>
+      <c r="F560" s="35"/>
+      <c r="G560" s="36"/>
+      <c r="H560" s="35"/>
+      <c r="I560" s="37"/>
+      <c r="J560" s="37"/>
+    </row>
+    <row r="561" spans="1:10">
+      <c r="A561" s="33" t="s">
+        <v>5085</v>
+      </c>
+      <c r="B561" s="38" t="s">
+        <v>5107</v>
+      </c>
+      <c r="C561" s="35"/>
+      <c r="D561" s="35"/>
+      <c r="E561" s="35"/>
+      <c r="F561" s="35"/>
+      <c r="G561" s="36"/>
+      <c r="H561" s="35"/>
+      <c r="I561" s="37"/>
+      <c r="J561" s="37"/>
+    </row>
+    <row r="562" spans="1:10">
+      <c r="A562" s="33" t="s">
+        <v>5086</v>
+      </c>
+      <c r="B562" s="34" t="s">
+        <v>5108</v>
+      </c>
+      <c r="C562" s="35"/>
+      <c r="D562" s="35"/>
+      <c r="E562" s="35"/>
+      <c r="F562" s="35"/>
+      <c r="G562" s="36"/>
+      <c r="H562" s="35"/>
+      <c r="I562" s="37"/>
+      <c r="J562" s="37"/>
+    </row>
+    <row r="563" spans="1:10">
+      <c r="A563" s="33" t="s">
+        <v>5087</v>
+      </c>
+      <c r="B563" s="34" t="s">
+        <v>5109</v>
+      </c>
+      <c r="C563" s="35"/>
+      <c r="D563" s="35"/>
+      <c r="E563" s="35"/>
+      <c r="F563" s="35"/>
+      <c r="G563" s="36"/>
+      <c r="H563" s="35"/>
+      <c r="I563" s="37"/>
+      <c r="J563" s="37"/>
+    </row>
+    <row r="564" spans="1:10">
+      <c r="A564" s="33" t="s">
+        <v>5088</v>
+      </c>
+      <c r="B564" s="34" t="s">
+        <v>5110</v>
+      </c>
+      <c r="C564" s="35"/>
+      <c r="D564" s="35"/>
+      <c r="E564" s="35"/>
+      <c r="F564" s="35"/>
+      <c r="G564" s="36"/>
+      <c r="H564" s="35"/>
+      <c r="I564" s="37"/>
+      <c r="J564" s="37"/>
+    </row>
+    <row r="565" spans="1:10">
+      <c r="A565" s="33" t="s">
+        <v>5089</v>
+      </c>
+      <c r="B565" s="34" t="s">
+        <v>5111</v>
+      </c>
+      <c r="C565" s="35"/>
+      <c r="D565" s="35"/>
+      <c r="E565" s="35"/>
+      <c r="F565" s="35"/>
+      <c r="G565" s="36"/>
+      <c r="H565" s="35"/>
+      <c r="I565" s="37"/>
+      <c r="J565" s="37"/>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
@@ -33485,6 +33999,15 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100F12BE0DB4A3DF641BF113FBF1C7EA261" ma:contentTypeVersion="16" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="c6b4b409d6b6c81c2874e5a51d11715e">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="43e153a8-5ef1-4f65-aac7-dc4685f18eaa" xmlns:ns3="6e0cf07b-8188-4b76-8f54-3cda03d37414" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="0521fade2ab7bf037697e8e8677cb864" ns2:_="" ns3:_="">
     <xsd:import namespace="43e153a8-5ef1-4f65-aac7-dc4685f18eaa"/>
@@ -33725,15 +34248,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9E20926E-9EFB-4B7E-90D4-905B08F8E59C}">
   <ds:schemaRefs>
@@ -33752,6 +34266,14 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{04FEE910-FEC8-48C6-9CF9-BF01BA5AD6FE}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C6201EF1-2938-4925-833A-11BB4654F7B4}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -33768,12 +34290,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{04FEE910-FEC8-48C6-9CF9-BF01BA5AD6FE}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Check for unique config name before saving to db.
</commit_message>
<xml_diff>
--- a/translations/translations.xlsx
+++ b/translations/translations.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/russell/Projects/GPS-Sample/translations/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{59A93F00-41D8-6846-BB2C-CF6E74189822}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{07D486B6-3C5F-544C-9611-6C8C84290E3C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="39520" yWindow="5180" windowWidth="29040" windowHeight="15720" xr2:uid="{C8C8ACD1-4E76-7942-B525-8D880B4ECA80}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17740" xr2:uid="{C8C8ACD1-4E76-7942-B525-8D880B4ECA80}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -67,7 +67,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5723" uniqueCount="5354">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5725" uniqueCount="5356">
   <si>
     <t>app_name</t>
   </si>
@@ -16129,13 +16129,19 @@
   </si>
   <si>
     <t>Allow Supervisors to edit this configuration.</t>
+  </si>
+  <si>
+    <t>name_already_exists</t>
+  </si>
+  <si>
+    <t>That configuration name already exists.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="19">
+  <fonts count="20">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -16257,6 +16263,12 @@
       <sz val="8"/>
       <color theme="1"/>
       <name val="Calibri Light (Headings)"/>
+    </font>
+    <font>
+      <sz val="9.8000000000000007"/>
+      <color rgb="FFBCBEC4"/>
+      <name val="JetBrains Mono"/>
+      <family val="3"/>
     </font>
   </fonts>
   <fills count="9">
@@ -16477,18 +16489,16 @@
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1" readingOrder="2"/>
     </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1" readingOrder="2"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -16710,8 +16720,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{73295AEA-8140-4EAB-A7A6-7D1875F4D7E7}" name="Table1" displayName="Table1" ref="A1:J582" totalsRowShown="0" headerRowDxfId="11" dataDxfId="10">
-  <autoFilter ref="A1:J582" xr:uid="{73295AEA-8140-4EAB-A7A6-7D1875F4D7E7}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{73295AEA-8140-4EAB-A7A6-7D1875F4D7E7}" name="Table1" displayName="Table1" ref="A1:J583" totalsRowShown="0" headerRowDxfId="11" dataDxfId="10">
+  <autoFilter ref="A1:J583" xr:uid="{73295AEA-8140-4EAB-A7A6-7D1875F4D7E7}"/>
   <tableColumns count="10">
     <tableColumn id="1" xr3:uid="{DE67F62A-9DCA-4DFE-8C98-83B024E5D946}" name="app_name" dataDxfId="9"/>
     <tableColumn id="2" xr3:uid="{BCDA3AB5-7BB5-4A21-ABBB-4186B52D559D}" name="GPSSample::en" dataDxfId="8"/>
@@ -17037,7 +17047,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8BD3E6CC-854C-5841-9577-D3ADD2982DB6}">
-  <dimension ref="A1:J582"/>
+  <dimension ref="A1:J583"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16"/>
   <cols>
     <col min="1" max="1" width="33.5" customWidth="1"/>
@@ -35291,196 +35301,212 @@
       </c>
     </row>
     <row r="571" spans="1:10">
-      <c r="A571" s="45" t="s">
+      <c r="A571" s="29" t="s">
         <v>5330</v>
       </c>
       <c r="B571" s="6" t="s">
         <v>5342</v>
       </c>
-      <c r="C571" s="47"/>
-      <c r="D571" s="47"/>
-      <c r="E571" s="47"/>
-      <c r="F571" s="47"/>
+      <c r="C571" s="9"/>
+      <c r="D571" s="9"/>
+      <c r="E571" s="9"/>
+      <c r="F571" s="9"/>
       <c r="G571" s="33"/>
-      <c r="H571" s="47"/>
-      <c r="I571" s="48"/>
-      <c r="J571" s="48"/>
+      <c r="H571" s="9"/>
+      <c r="I571" s="12"/>
+      <c r="J571" s="12"/>
     </row>
     <row r="572" spans="1:10">
-      <c r="A572" s="45" t="s">
+      <c r="A572" s="29" t="s">
         <v>5331</v>
       </c>
-      <c r="B572" s="46" t="s">
+      <c r="B572" s="27" t="s">
         <v>5343</v>
       </c>
-      <c r="C572" s="47"/>
-      <c r="D572" s="47"/>
-      <c r="E572" s="47"/>
-      <c r="F572" s="47"/>
+      <c r="C572" s="9"/>
+      <c r="D572" s="9"/>
+      <c r="E572" s="9"/>
+      <c r="F572" s="9"/>
       <c r="G572" s="33"/>
-      <c r="H572" s="47"/>
-      <c r="I572" s="48"/>
-      <c r="J572" s="48"/>
+      <c r="H572" s="9"/>
+      <c r="I572" s="12"/>
+      <c r="J572" s="12"/>
     </row>
     <row r="573" spans="1:10">
-      <c r="A573" s="45" t="s">
+      <c r="A573" s="29" t="s">
         <v>5332</v>
       </c>
-      <c r="B573" s="50" t="s">
+      <c r="B573" s="46" t="s">
         <v>5344</v>
       </c>
-      <c r="C573" s="47"/>
-      <c r="D573" s="47"/>
-      <c r="E573" s="47"/>
-      <c r="F573" s="47"/>
+      <c r="C573" s="9"/>
+      <c r="D573" s="9"/>
+      <c r="E573" s="9"/>
+      <c r="F573" s="9"/>
       <c r="G573" s="33"/>
-      <c r="H573" s="47"/>
-      <c r="I573" s="48"/>
-      <c r="J573" s="48"/>
+      <c r="H573" s="9"/>
+      <c r="I573" s="12"/>
+      <c r="J573" s="12"/>
     </row>
     <row r="574" spans="1:10">
-      <c r="A574" s="45" t="s">
+      <c r="A574" s="29" t="s">
         <v>5333</v>
       </c>
-      <c r="B574" s="46" t="s">
+      <c r="B574" s="27" t="s">
         <v>5345</v>
       </c>
-      <c r="C574" s="47"/>
-      <c r="D574" s="47"/>
-      <c r="E574" s="47"/>
-      <c r="F574" s="47"/>
+      <c r="C574" s="9"/>
+      <c r="D574" s="9"/>
+      <c r="E574" s="9"/>
+      <c r="F574" s="9"/>
       <c r="G574" s="33"/>
-      <c r="H574" s="47"/>
-      <c r="I574" s="48"/>
-      <c r="J574" s="48"/>
+      <c r="H574" s="9"/>
+      <c r="I574" s="12"/>
+      <c r="J574" s="12"/>
     </row>
     <row r="575" spans="1:10">
-      <c r="A575" s="45" t="s">
+      <c r="A575" s="29" t="s">
         <v>5334</v>
       </c>
-      <c r="B575" s="50" t="s">
+      <c r="B575" s="46" t="s">
         <v>5346</v>
       </c>
-      <c r="C575" s="47"/>
-      <c r="D575" s="47"/>
-      <c r="E575" s="47"/>
-      <c r="F575" s="47"/>
+      <c r="C575" s="9"/>
+      <c r="D575" s="9"/>
+      <c r="E575" s="9"/>
+      <c r="F575" s="9"/>
       <c r="G575" s="33"/>
-      <c r="H575" s="47"/>
-      <c r="I575" s="48"/>
-      <c r="J575" s="48"/>
+      <c r="H575" s="9"/>
+      <c r="I575" s="12"/>
+      <c r="J575" s="12"/>
     </row>
     <row r="576" spans="1:10">
-      <c r="A576" s="45" t="s">
+      <c r="A576" s="29" t="s">
         <v>5335</v>
       </c>
-      <c r="B576" s="46" t="s">
+      <c r="B576" s="27" t="s">
         <v>5347</v>
       </c>
-      <c r="C576" s="47"/>
-      <c r="D576" s="47"/>
-      <c r="E576" s="47"/>
-      <c r="F576" s="47"/>
+      <c r="C576" s="9"/>
+      <c r="D576" s="9"/>
+      <c r="E576" s="9"/>
+      <c r="F576" s="9"/>
       <c r="G576" s="33"/>
-      <c r="H576" s="47"/>
-      <c r="I576" s="48"/>
-      <c r="J576" s="48"/>
+      <c r="H576" s="9"/>
+      <c r="I576" s="12"/>
+      <c r="J576" s="12"/>
     </row>
     <row r="577" spans="1:10">
-      <c r="A577" s="45" t="s">
+      <c r="A577" s="29" t="s">
         <v>5336</v>
       </c>
-      <c r="B577" s="46" t="s">
+      <c r="B577" s="27" t="s">
         <v>5348</v>
       </c>
-      <c r="C577" s="47"/>
-      <c r="D577" s="47"/>
-      <c r="E577" s="47"/>
-      <c r="F577" s="47"/>
+      <c r="C577" s="9"/>
+      <c r="D577" s="9"/>
+      <c r="E577" s="9"/>
+      <c r="F577" s="9"/>
       <c r="G577" s="33"/>
-      <c r="H577" s="47"/>
-      <c r="I577" s="48"/>
-      <c r="J577" s="48"/>
+      <c r="H577" s="9"/>
+      <c r="I577" s="12"/>
+      <c r="J577" s="12"/>
     </row>
     <row r="578" spans="1:10">
-      <c r="A578" s="45" t="s">
+      <c r="A578" s="29" t="s">
         <v>5337</v>
       </c>
-      <c r="B578" s="46" t="s">
+      <c r="B578" s="27" t="s">
         <v>5349</v>
       </c>
-      <c r="C578" s="47"/>
-      <c r="D578" s="47"/>
-      <c r="E578" s="47"/>
-      <c r="F578" s="47"/>
+      <c r="C578" s="9"/>
+      <c r="D578" s="9"/>
+      <c r="E578" s="9"/>
+      <c r="F578" s="9"/>
       <c r="G578" s="33"/>
-      <c r="H578" s="47"/>
-      <c r="I578" s="48"/>
-      <c r="J578" s="48"/>
+      <c r="H578" s="9"/>
+      <c r="I578" s="12"/>
+      <c r="J578" s="12"/>
     </row>
     <row r="579" spans="1:10">
-      <c r="A579" s="45" t="s">
+      <c r="A579" s="29" t="s">
         <v>5338</v>
       </c>
-      <c r="B579" s="50" t="s">
+      <c r="B579" s="46" t="s">
         <v>5350</v>
       </c>
-      <c r="C579" s="47"/>
-      <c r="D579" s="47"/>
-      <c r="E579" s="47"/>
-      <c r="F579" s="47"/>
+      <c r="C579" s="9"/>
+      <c r="D579" s="9"/>
+      <c r="E579" s="9"/>
+      <c r="F579" s="9"/>
       <c r="G579" s="33"/>
-      <c r="H579" s="47"/>
-      <c r="I579" s="48"/>
-      <c r="J579" s="48"/>
+      <c r="H579" s="9"/>
+      <c r="I579" s="12"/>
+      <c r="J579" s="12"/>
     </row>
     <row r="580" spans="1:10" ht="25">
-      <c r="A580" s="45" t="s">
+      <c r="A580" s="29" t="s">
         <v>5339</v>
       </c>
-      <c r="B580" s="46" t="s">
+      <c r="B580" s="27" t="s">
         <v>5351</v>
       </c>
-      <c r="C580" s="47"/>
-      <c r="D580" s="47"/>
-      <c r="E580" s="47"/>
-      <c r="F580" s="47"/>
+      <c r="C580" s="9"/>
+      <c r="D580" s="9"/>
+      <c r="E580" s="9"/>
+      <c r="F580" s="9"/>
       <c r="G580" s="33"/>
-      <c r="H580" s="47"/>
-      <c r="I580" s="48"/>
-      <c r="J580" s="48"/>
+      <c r="H580" s="9"/>
+      <c r="I580" s="12"/>
+      <c r="J580" s="12"/>
     </row>
     <row r="581" spans="1:10">
-      <c r="A581" s="45" t="s">
+      <c r="A581" s="29" t="s">
         <v>5340</v>
       </c>
-      <c r="B581" s="49" t="s">
+      <c r="B581" s="45" t="s">
         <v>5352</v>
       </c>
-      <c r="C581" s="47"/>
-      <c r="D581" s="47"/>
-      <c r="E581" s="47"/>
-      <c r="F581" s="47"/>
+      <c r="C581" s="9"/>
+      <c r="D581" s="9"/>
+      <c r="E581" s="9"/>
+      <c r="F581" s="9"/>
       <c r="G581" s="33"/>
-      <c r="H581" s="47"/>
-      <c r="I581" s="48"/>
-      <c r="J581" s="48"/>
+      <c r="H581" s="9"/>
+      <c r="I581" s="12"/>
+      <c r="J581" s="12"/>
     </row>
     <row r="582" spans="1:10">
-      <c r="A582" s="45" t="s">
+      <c r="A582" s="29" t="s">
         <v>5341</v>
       </c>
-      <c r="B582" s="46" t="s">
+      <c r="B582" s="27" t="s">
         <v>5353</v>
       </c>
-      <c r="C582" s="47"/>
-      <c r="D582" s="47"/>
-      <c r="E582" s="47"/>
-      <c r="F582" s="47"/>
+      <c r="C582" s="9"/>
+      <c r="D582" s="9"/>
+      <c r="E582" s="9"/>
+      <c r="F582" s="9"/>
       <c r="G582" s="33"/>
-      <c r="H582" s="47"/>
-      <c r="I582" s="48"/>
-      <c r="J582" s="48"/>
+      <c r="H582" s="9"/>
+      <c r="I582" s="12"/>
+      <c r="J582" s="12"/>
+    </row>
+    <row r="583" spans="1:10">
+      <c r="A583" s="47" t="s">
+        <v>5354</v>
+      </c>
+      <c r="B583" s="50" t="s">
+        <v>5355</v>
+      </c>
+      <c r="C583" s="48"/>
+      <c r="D583" s="48"/>
+      <c r="E583" s="48"/>
+      <c r="F583" s="48"/>
+      <c r="G583" s="33"/>
+      <c r="H583" s="48"/>
+      <c r="I583" s="49"/>
+      <c r="J583" s="49"/>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
@@ -35494,14 +35520,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="6e0cf07b-8188-4b76-8f54-3cda03d37414" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="43e153a8-5ef1-4f65-aac7-dc4685f18eaa">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -35746,27 +35770,20 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="6e0cf07b-8188-4b76-8f54-3cda03d37414" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="43e153a8-5ef1-4f65-aac7-dc4685f18eaa">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9E20926E-9EFB-4B7E-90D4-905B08F8E59C}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{04FEE910-FEC8-48C6-9CF9-BF01BA5AD6FE}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="6e0cf07b-8188-4b76-8f54-3cda03d37414"/>
-    <ds:schemaRef ds:uri="43e153a8-5ef1-4f65-aac7-dc4685f18eaa"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -35791,9 +35808,18 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{04FEE910-FEC8-48C6-9CF9-BF01BA5AD6FE}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9E20926E-9EFB-4B7E-90D4-905B08F8E59C}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="6e0cf07b-8188-4b76-8f54-3cda03d37414"/>
+    <ds:schemaRef ds:uri="43e153a8-5ef1-4f65-aac7-dc4685f18eaa"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>